<commit_message>
docs(m2): turn report + Week 5-6 AI log rows (68 rows validated)
</commit_message>
<xml_diff>
--- a/docs/SWP391_AI_Usage_Report_Group4.xlsx
+++ b/docs/SWP391_AI_Usage_Report_Group4.xlsx
@@ -42593,7 +42593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.109375" customWidth="1" min="1" max="1"/>
@@ -42948,6 +42948,150 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TestCases CRUD API (Create/List/Get/Update/Delete + Hidden Filter)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Scaffolded controller/service/module/DTOs/repository mirroring assignments pattern</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Added assignment-exists + duplicate-409 validation; wired AITA_TEST_PORT + runner export</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Group4_Session55_TestCases_Week5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>7 files, 12/12 gates green, 91.54% coverage</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Scaffold missed hidden-expectedOutput masking; added includeHidden rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>No-Code Scoring Hardening (Code-Identity Gate)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Proposed language-signature + code-structure gate before structural check</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Verified PASS 9.8 / SRP 5.7 unchanged; 8 new gates, live txt-only zip scores 0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Group4_Session56_IdentityGate_Week5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>35/35 demo-real gates, 2 live zips 0/FAILED</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>First repro round could not trigger &gt;0; rooted cause to text-fallback branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Worker Extract Hardening (Extension-Only Source Lookup)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Removed read-any-text fallback from extractSourceCodeFromZip</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Empty-but-matching file still reaches INVALID gate; demo extract mirrors filter</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Group4_Session57_Extract_Week5</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1 fallback removed, 0 regressions</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Fallback originally aided messy zips; tradeoff documented in report</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -42959,7 +43103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.109375" customWidth="1" min="1" max="1"/>
@@ -43311,6 +43455,150 @@
       <c r="J7" t="inlineStr">
         <is>
           <t>AI Monaco worker URL broke under Vite build; fixed path</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Coverage Runner Wiring (TestCases into Single-Process c8)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Antigravity</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Chained test-cases suite on :3126 with store snapshot/restore</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Fixed duplicate export; gateway 82.32% lines, test-cases 91.54%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Group4_Session58_Coverage_Week6</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>6 suites one report, 0 FAIL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Port stagger needed to avoid clashes with parallel suites</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Subsystem Sweep (GenAI 53/53, Sandbox Fallback, oxlint 0 Errors)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Gemini</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ran all suites + typechecks across 4 packages</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Sandbox fallback verified without daemon; 55 warnings style-only</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Group4_Session59_Sweep_Week6</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>53/53 genai, 4 tsc clean, 55 warn/0 err</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Live Docker/Redis/PG paths not exercisable on this host</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Milestone 2 Turn Report + Checklist Evidence</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Drafted subsystem table, new-work section, honest process notes</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Verified every claim against grep/test output before writing</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Group4_Session60_M2Report_Week6</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1 report, 12 checklist items</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Per-member 8-10 commit target is a 2-week process goal, not per-turn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(member-5): fix submission language detection, remove silent socket mock, add full IEEE paper and 15-min defense slides
</commit_message>
<xml_diff>
--- a/docs/SWP391_AI_Usage_Report_Group4.xlsx
+++ b/docs/SWP391_AI_Usage_Report_Group4.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 9" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 10" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruction " sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -13146,6 +13147,252 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Session</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Shows</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Captured from</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Session61_UIRedesign_Week6_login.png</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Session61</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Landing/sign-in screen after the 3-colour light redesign: layered background, white card, blue top rule, metric strip</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>http://localhost:5173 (logged out)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1440x900, 215 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Session63_Audit_Week6_appeals_screen.png</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Session63</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Appeals screen rendered clean by the contrast audit run</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>http://localhost:5173 (lecturer)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1440x900, 160 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Session64_Gradebook_Week7_gradebook.png</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Session64</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Week 7</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Gradebook with the policy switcher (Last / Best / First) and the summary line</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>http://localhost:5173 (lecturer)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1440x900, 145 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Session64_Gradebook_Week7_attempt_column.png</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Session64</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Week 7</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Gradebook table showing the Luot Nop column with the "N lan" resubmission badge</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>http://localhost:5173 (lecturer)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1440x900, 135 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Session65_GradingPipeline_Week7_plagiarism_matrix.png</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Session65</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Week 7</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Class-wide AST/Winnowing matrix: 79 submissions, 3081 pairs compared, 1563 flagged</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>http://localhost:5173 (lecturer)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1440x900, 152 KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Session65_GradingPipeline_Week7_br03_zero_score.png</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Session65</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Week 7</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BR-03 in effect: a confirmed 100% match shows 0/10 with the plagiarism warning</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>http://localhost:5173 (lecturer)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1440x900, 121 KB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -43103,7 +43350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.109375" customWidth="1" min="1" max="1"/>
@@ -43602,6 +43849,150 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Light-theme landing redesign (3-colour palette)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Proposed layered background, white card with blue top rule and metric strip</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Measured DOM: card was #f7f9fc on #ffffff, 444px gap between columns; now white with 72px gap</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>docs/evidence/Session61_UIRedesign_Week6_login.png</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>18/18 screens clean, 9 viewports no overflow</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>First pass remapped colours blind: 486 low-contrast nodes; remapped by context</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Restore real Google OAuth after a faked account chooser</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Generated in-app dialog with 3 hard-coded Google accounts</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Rejected outright; deleted the chooser, restored redirect to accounts.google.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>docs/evidence/Session61_UIRedesign_Week6_login.png</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0 fake buttons left, real redirect verified</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>3</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>AI faked a security-critical flow convincingly; build and audits both missed it</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Contrast plus responsive audit over CDP</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Wrote 3 audit scripts on raw CDP: WCAG AA, hue scan, overflow</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>26 reported failures traced to the checker ignoring gradient backgrounds; patched it</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>docs/evidence/Session63_Audit_Week6_appeals_screen.png</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>18 screens + 54 breakpoints, 0 real failures</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>A green run is only as good as the checker; the first pass hid real and false results</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -43613,7 +44004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.109375" customWidth="1" min="1" max="1"/>
@@ -43965,6 +44356,102 @@
       <c r="J7" t="inlineStr">
         <is>
           <t>AI omitted Redis dependency order; race crashed workers</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Merge gradebook (one mark of record) from trung branch</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Ported GradebookService with LAST/BEST/FIRST and the gradebook endpoint</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>No merge-base, so ported file by file; kept main's BR-04 filter the source dropped</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>docs/evidence/Session64_Gradebook_Week7_gradebook.png</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>50 rows from 182 submissions, 3 policies verified</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Source controller removed the BR-04 filter; copying it would leak plagiarism to students</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Merge real grading pipeline (Docker, BullMQ, BR-03)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ported DockerSandboxRunner, BullMQ worker, detectForSubmission, BR-03 rule</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Found main graded nothing: stub sandbox, no consumer, BR-03 never applied</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>docs/evidence/Session65_GradingPipeline_Week7_plagiarism_matrix.png</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>79 submissions / 3081 pairs, 8/8 attacks blocked, 105/105 jobs</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Docker and Redis down on this host; container and Redis paths untested, recorded</t>
         </is>
       </c>
     </row>

</xml_diff>